<commit_message>
fixed password issue so now special characters are allowed
</commit_message>
<xml_diff>
--- a/Audit_Code/public/ISO_SOA_A5.xlsx
+++ b/Audit_Code/public/ISO_SOA_A5.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ab\Desktop\Compliance\Audit_Code\public\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Documents\Compliance\Audit_Code\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -14,7 +14,7 @@
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="152511"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -236,15 +236,9 @@
     <t>Records shall be protected from loss, destruction, falsification, unau thorized access and unauthorized release.</t>
   </si>
   <si>
-    <t>Privacy and protection of person- al identifiable information (PII)</t>
-  </si>
-  <si>
     <t>The organization shall identify and meet the requirements regarding the preservation of privacy and protection of PII according to applicable laws and regulations and contractual requirements.</t>
   </si>
   <si>
-    <t>Independent review of informa- tion security</t>
-  </si>
-  <si>
     <t>The organization’s approach to managing information security and its implementation including people, processes and technologies shall be reviewed independently at planned intervals, or when significant changes occur.</t>
   </si>
   <si>
@@ -258,12 +252,18 @@
   </si>
   <si>
     <t>Operating procedures for information processing facilities shall be documented and made available to personnel who need them.</t>
+  </si>
+  <si>
+    <t>Privacy and protection of personal identifiable information (PII)</t>
+  </si>
+  <si>
+    <t>Independent review of information security</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -1007,10 +1007,10 @@
         <v>5.34</v>
       </c>
       <c r="B35" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="C35" s="8" t="s">
         <v>70</v>
-      </c>
-      <c r="C35" s="8" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="36" spans="1:3" ht="42.75" x14ac:dyDescent="0.25">
@@ -1018,10 +1018,10 @@
         <v>5.35</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="C36" s="8" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
     </row>
     <row r="37" spans="1:3" ht="28.5" x14ac:dyDescent="0.25">
@@ -1029,10 +1029,10 @@
         <v>5.36</v>
       </c>
       <c r="B37" s="5" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C37" s="8" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="38" spans="1:3" ht="28.5" x14ac:dyDescent="0.25">
@@ -1040,10 +1040,10 @@
         <v>5.37</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C38" s="8" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
   </sheetData>

</xml_diff>